<commit_message>
fix(backlink): parse 2025/2026 Excel formats (plain HKD, hkd suffix, serial dates)
- Support cost values like 409, 359 hkd without dollar sign
- Parse Excel serial dates in date columns (e.g. 46175)
- Re-import: 73 paid records across 2024-2026 (was 37 x 2024 only)
- Update source Excel workbook

Co-authored-by: chifung-BWSolution <chifung-BWSolution@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/SEO backlink order record + keywords update schedule.xlsx
+++ b/data/SEO backlink order record + keywords update schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBD26FE0-9E1C-4814-9F95-B8A660862CFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DA178DF-286A-4E99-B87C-99C5DFD22B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="175">
   <si>
     <t>Brand</t>
   </si>
@@ -35,12 +35,6 @@
   </si>
   <si>
     <t>Domain</t>
-  </si>
-  <si>
-    <t>Google Ads</t>
-  </si>
-  <si>
-    <t>Website Platform Link</t>
   </si>
   <si>
     <t>Feb</t>
@@ -97,9 +91,6 @@
     <t>FCC</t>
   </si>
   <si>
-    <t>https://www.victoria-beauty.com/</t>
-  </si>
-  <si>
     <t xml:space="preserve">Wine Passions </t>
   </si>
   <si>
@@ -116,14 +107,6 @@
   </si>
   <si>
     <t>https://hkofficedesign.com/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A1 BSC Victoria-Beauty.com
-318-489-6707
-</t>
-  </si>
-  <si>
-    <t>https://admin.shopify.com/store/victoria-beauty-7843?no_redirect=true</t>
   </si>
   <si>
     <t>23/11</t>
@@ -251,9 +234,6 @@
   </si>
   <si>
     <t>BW Furniture</t>
-  </si>
-  <si>
-    <t>https://admin.shopify.com/store/beauty100-magazine?no_redirect=true</t>
   </si>
   <si>
     <t>BW Furniture 辦公室傢俬</t>
@@ -588,11 +568,15 @@
   </si>
   <si>
     <t>Domain</t>
-    <phoneticPr fontId="21" type="noConversion"/>
+    <phoneticPr fontId="20" type="noConversion"/>
   </si>
   <si>
     <t>Nov</t>
-    <phoneticPr fontId="21" type="noConversion"/>
+    <phoneticPr fontId="20" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.attitude-beauty.com/</t>
+    <phoneticPr fontId="20" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -699,12 +683,6 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0563C1"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -742,6 +720,13 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -766,8 +751,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -802,17 +788,18 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="177" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="176" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="176" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="超連結" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1118,7 +1105,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>228600</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>9525</xdr:rowOff>
@@ -1389,37 +1376,37 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="2">
         <v>2024</v>
       </c>
-      <c r="G1" s="29" t="s">
-        <v>179</v>
+      <c r="G1" s="28" t="s">
+        <v>173</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I1" s="1"/>
       <c r="J1" s="8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L1" s="1"/>
       <c r="M1" s="2">
         <v>2025</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Q1" s="1"/>
       <c r="R1" s="10"/>
@@ -1428,23 +1415,23 @@
         <v>2026</v>
       </c>
       <c r="U1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="W1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="W1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="X1" s="3" t="s">
-        <v>9</v>
       </c>
       <c r="Y1" s="1"/>
       <c r="Z1" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AA1" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="AB1" s="1"/>
       <c r="AC1" s="1"/>
@@ -1471,44 +1458,44 @@
     </row>
     <row r="2" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>30</v>
-      </c>
       <c r="E2" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F2" s="11"/>
       <c r="G2" s="11" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="I2" s="11"/>
       <c r="J2" s="16">
         <v>45455</v>
       </c>
       <c r="K2" s="11" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="L2" s="11"/>
       <c r="M2" s="11"/>
       <c r="N2" s="11" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="O2" s="20">
         <v>409</v>
       </c>
       <c r="P2" s="11" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="Q2" s="11"/>
       <c r="R2" s="11"/>
@@ -1524,11 +1511,11 @@
         <v>677.53</v>
       </c>
       <c r="X2" s="11" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="Y2" s="11"/>
       <c r="Z2" s="11" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="AA2" s="11"/>
       <c r="AB2" s="11"/>
@@ -1556,33 +1543,33 @@
     </row>
     <row r="3" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F3" s="11"/>
       <c r="G3" s="11" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="I3" s="11"/>
       <c r="J3" s="16">
         <v>45455</v>
       </c>
       <c r="K3" s="11" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="L3" s="11"/>
       <c r="M3" s="11"/>
@@ -1627,33 +1614,33 @@
     </row>
     <row r="4" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F4" s="11"/>
       <c r="G4" s="11" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="I4" s="11"/>
       <c r="J4" s="16">
         <v>45455</v>
       </c>
       <c r="K4" s="11" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="L4" s="11"/>
       <c r="M4" s="11"/>
@@ -1698,33 +1685,33 @@
     </row>
     <row r="5" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F5" s="11"/>
       <c r="G5" s="11" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="I5" s="11"/>
       <c r="J5" s="16">
         <v>45455</v>
       </c>
       <c r="K5" s="11" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="L5" s="11"/>
       <c r="M5" s="11"/>
@@ -1769,19 +1756,19 @@
     </row>
     <row r="6" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F6" s="11"/>
       <c r="G6" s="11"/>
@@ -1791,7 +1778,7 @@
         <v>45363</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="L6" s="11"/>
       <c r="M6" s="11"/>
@@ -1836,19 +1823,19 @@
     </row>
     <row r="7" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F7" s="11"/>
       <c r="G7" s="11"/>
@@ -1858,7 +1845,7 @@
         <v>45394</v>
       </c>
       <c r="K7" s="11" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="L7" s="11"/>
       <c r="M7" s="11"/>
@@ -1903,33 +1890,33 @@
     </row>
     <row r="8" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F8" s="11"/>
       <c r="G8" s="11" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="I8" s="11"/>
       <c r="J8" s="16">
         <v>45455</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="L8" s="11"/>
       <c r="M8" s="11"/>
@@ -1974,33 +1961,33 @@
     </row>
     <row r="9" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F9" s="11"/>
       <c r="G9" s="11" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="I9" s="11"/>
       <c r="J9" s="16">
         <v>45455</v>
       </c>
       <c r="K9" s="11" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="L9" s="11"/>
       <c r="M9" s="11"/>
@@ -2045,19 +2032,19 @@
     </row>
     <row r="10" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F10" s="11"/>
       <c r="G10" s="11"/>
@@ -2067,7 +2054,7 @@
         <v>45363</v>
       </c>
       <c r="K10" s="11" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="L10" s="11"/>
       <c r="M10" s="11"/>
@@ -2112,19 +2099,19 @@
     </row>
     <row r="11" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B11" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="C11" s="9" t="s">
-        <v>105</v>
-      </c>
       <c r="D11" s="15" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F11" s="11"/>
       <c r="G11" s="11"/>
@@ -2134,7 +2121,7 @@
         <v>45394</v>
       </c>
       <c r="K11" s="11" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
@@ -2179,19 +2166,19 @@
     </row>
     <row r="12" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F12" s="11"/>
       <c r="G12" s="11"/>
@@ -2242,19 +2229,19 @@
     </row>
     <row r="13" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F13" s="11"/>
       <c r="G13" s="11"/>
@@ -2305,19 +2292,19 @@
     </row>
     <row r="14" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F14" s="11"/>
       <c r="G14" s="11"/>
@@ -2368,19 +2355,19 @@
     </row>
     <row r="15" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
-      <c r="D15" s="27" t="s">
-        <v>115</v>
+      <c r="D15" s="26" t="s">
+        <v>109</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F15" s="11"/>
       <c r="G15" s="11"/>
@@ -2431,19 +2418,19 @@
     </row>
     <row r="16" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F16" s="11"/>
       <c r="G16" s="11"/>
@@ -2494,19 +2481,19 @@
     </row>
     <row r="17" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F17" s="11"/>
       <c r="G17" s="11"/>
@@ -2557,19 +2544,19 @@
     </row>
     <row r="18" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F18" s="11"/>
       <c r="G18" s="11"/>
@@ -2579,7 +2566,7 @@
         <v>45363</v>
       </c>
       <c r="K18" s="11" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="L18" s="11"/>
       <c r="M18" s="11"/>
@@ -2624,33 +2611,33 @@
     </row>
     <row r="19" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
-      <c r="D19" s="28" t="s">
-        <v>124</v>
+      <c r="D19" s="27" t="s">
+        <v>118</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F19" s="11"/>
       <c r="G19" s="11" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="I19" s="11"/>
       <c r="J19" s="16">
         <v>45455</v>
       </c>
       <c r="K19" s="11" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="L19" s="11"/>
       <c r="M19" s="11"/>
@@ -2693,19 +2680,19 @@
     </row>
     <row r="20" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B20" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>126</v>
+      <c r="C20" s="9" t="s">
+        <v>121</v>
       </c>
-      <c r="C20" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="D20" s="27" t="s">
-        <v>128</v>
+      <c r="D20" s="26" t="s">
+        <v>122</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F20" s="11"/>
       <c r="G20" s="11"/>
@@ -2715,7 +2702,7 @@
         <v>45394</v>
       </c>
       <c r="K20" s="11" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="L20" s="11"/>
       <c r="M20" s="11"/>
@@ -2758,19 +2745,19 @@
     </row>
     <row r="21" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
-      <c r="D21" s="27" t="s">
-        <v>130</v>
+      <c r="D21" s="26" t="s">
+        <v>124</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F21" s="11"/>
       <c r="G21" s="11"/>
@@ -2780,7 +2767,7 @@
         <v>45363</v>
       </c>
       <c r="K21" s="11" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="L21" s="11"/>
       <c r="M21" s="11"/>
@@ -2823,19 +2810,19 @@
     </row>
     <row r="22" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="B22" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="C22" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="C22" s="9" t="s">
-        <v>132</v>
-      </c>
       <c r="D22" s="17" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F22" s="11"/>
       <c r="G22" s="11"/>
@@ -2845,7 +2832,7 @@
         <v>45394</v>
       </c>
       <c r="K22" s="11" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="L22" s="11"/>
       <c r="M22" s="11"/>
@@ -2888,19 +2875,19 @@
     </row>
     <row r="23" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
-      <c r="D23" s="27" t="s">
-        <v>136</v>
+      <c r="D23" s="26" t="s">
+        <v>130</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F23" s="11"/>
       <c r="G23" s="11"/>
@@ -2949,19 +2936,19 @@
     </row>
     <row r="24" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
-      <c r="D24" s="27" t="s">
-        <v>138</v>
+      <c r="D24" s="26" t="s">
+        <v>132</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F24" s="11"/>
       <c r="G24" s="11"/>
@@ -3010,19 +2997,19 @@
     </row>
     <row r="25" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
-      <c r="D25" s="27" t="s">
-        <v>141</v>
+      <c r="D25" s="26" t="s">
+        <v>135</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F25" s="11"/>
       <c r="G25" s="11"/>
@@ -3071,19 +3058,19 @@
     </row>
     <row r="26" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F26" s="11"/>
       <c r="G26" s="11"/>
@@ -3110,7 +3097,7 @@
         <v>547.73</v>
       </c>
       <c r="X26" s="11" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="Y26" s="11"/>
       <c r="Z26" s="11"/>
@@ -3140,19 +3127,19 @@
     </row>
     <row r="27" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
-      <c r="D27" s="27" t="s">
-        <v>146</v>
+      <c r="D27" s="26" t="s">
+        <v>140</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F27" s="11"/>
       <c r="G27" s="11"/>
@@ -3201,19 +3188,19 @@
     </row>
     <row r="28" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
-      <c r="D28" s="27" t="s">
-        <v>148</v>
+      <c r="D28" s="26" t="s">
+        <v>142</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F28" s="11"/>
       <c r="G28" s="11"/>
@@ -3262,19 +3249,19 @@
     </row>
     <row r="29" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
-      <c r="D29" s="27" t="s">
-        <v>150</v>
+      <c r="D29" s="26" t="s">
+        <v>144</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F29" s="11"/>
       <c r="G29" s="11"/>
@@ -3323,26 +3310,26 @@
     </row>
     <row r="30" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
-      <c r="D30" s="27" t="s">
-        <v>152</v>
+      <c r="D30" s="26" t="s">
+        <v>146</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F30" s="11"/>
       <c r="G30" s="11" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="H30" s="11" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="I30" s="11"/>
       <c r="J30" s="16"/>
@@ -3388,19 +3375,19 @@
     </row>
     <row r="31" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
-      <c r="D31" s="27" t="s">
-        <v>155</v>
+      <c r="D31" s="26" t="s">
+        <v>149</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F31" s="11"/>
       <c r="G31" s="11"/>
@@ -3449,19 +3436,19 @@
     </row>
     <row r="32" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
-      <c r="D32" s="27" t="s">
-        <v>157</v>
+      <c r="D32" s="26" t="s">
+        <v>151</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F32" s="11"/>
       <c r="G32" s="11"/>
@@ -3510,19 +3497,19 @@
     </row>
     <row r="33" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A33" s="9" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
-      <c r="D33" s="27" t="s">
-        <v>159</v>
+      <c r="D33" s="26" t="s">
+        <v>153</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F33" s="11"/>
       <c r="G33" s="11"/>
@@ -3571,19 +3558,19 @@
     </row>
     <row r="34" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F34" s="11"/>
       <c r="G34" s="11"/>
@@ -3632,19 +3619,19 @@
     </row>
     <row r="35" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F35" s="11"/>
       <c r="G35" s="11"/>
@@ -3693,19 +3680,19 @@
     </row>
     <row r="36" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F36" s="11"/>
       <c r="G36" s="11"/>
@@ -3754,19 +3741,19 @@
     </row>
     <row r="37" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F37" s="11"/>
       <c r="G37" s="11"/>
@@ -3815,19 +3802,19 @@
     </row>
     <row r="38" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F38" s="11"/>
       <c r="G38" s="11"/>
@@ -3854,11 +3841,11 @@
         <v>374.72</v>
       </c>
       <c r="X38" s="11" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="Y38" s="11"/>
       <c r="Z38" s="11" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="AA38" s="11"/>
       <c r="AB38" s="11"/>
@@ -3886,19 +3873,19 @@
     </row>
     <row r="39" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A39" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F39" s="11"/>
       <c r="G39" s="11"/>
@@ -3947,19 +3934,19 @@
     </row>
     <row r="40" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F40" s="11"/>
       <c r="G40" s="11"/>
@@ -3978,7 +3965,7 @@
       <c r="T40" s="11"/>
       <c r="U40" s="11"/>
       <c r="V40" s="11"/>
-      <c r="W40" s="25"/>
+      <c r="W40" s="24"/>
       <c r="X40" s="11"/>
       <c r="Y40" s="11"/>
       <c r="Z40" s="11"/>
@@ -4008,19 +3995,19 @@
     </row>
     <row r="41" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F41" s="11"/>
       <c r="G41" s="11"/>
@@ -53385,7 +53372,7 @@
       <c r="AW1008" s="11"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="21" type="noConversion"/>
+  <phoneticPr fontId="20" type="noConversion"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B41" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"1. 主要,2. 次要,3. side - 主要,4. side - 次要,5. 沒有重要,6. 其它業務"</formula1>
@@ -53475,41 +53462,41 @@
         <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E1" s="4">
         <v>2024</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H1" s="5"/>
       <c r="I1" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="N1" s="8">
         <v>2025</v>
       </c>
       <c r="O1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="P1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="P1" s="6" t="s">
-        <v>8</v>
-      </c>
       <c r="Q1" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="T1" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="U1" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V1" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Y1" s="6"/>
       <c r="Z1" s="6"/>
@@ -53517,72 +53504,72 @@
         <v>2026</v>
       </c>
       <c r="AB1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="AC1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="AD1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AE1" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="AD1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="AE1" s="3" t="s">
-        <v>9</v>
       </c>
       <c r="AF1" s="1"/>
       <c r="AG1" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AH1" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="AI1" s="6"/>
       <c r="AJ1" s="6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:36" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D2" s="11"/>
       <c r="E2" s="11"/>
       <c r="F2" s="11" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="H2" s="16"/>
       <c r="I2" s="16">
         <v>45455</v>
       </c>
       <c r="J2" s="11" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="N2" s="11"/>
       <c r="O2" s="11" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="P2" s="11" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="Q2" s="11" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="T2" s="11" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="U2" s="11" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="V2" s="11" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="AA2" s="11"/>
       <c r="AB2" s="11"/>
@@ -53594,197 +53581,197 @@
     </row>
     <row r="3" spans="1:36" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D3" s="11"/>
       <c r="E3" s="6"/>
       <c r="F3" s="6" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="H3" s="16"/>
       <c r="I3" s="16">
         <v>45455</v>
       </c>
       <c r="J3" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC3" s="24">
         <v>46</v>
       </c>
-      <c r="AD3" s="25"/>
+      <c r="AC3" s="23">
+        <v>46</v>
+      </c>
+      <c r="AD3" s="24"/>
     </row>
     <row r="4" spans="1:36" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="D4" s="11"/>
-      <c r="AB4" s="26">
+      <c r="AB4" s="25">
         <v>46175</v>
       </c>
-      <c r="AC4" s="24">
+      <c r="AC4" s="23">
         <v>34</v>
       </c>
-      <c r="AD4" s="25">
+      <c r="AD4" s="24">
         <v>374.72</v>
       </c>
       <c r="AE4" s="6" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AG4" s="6" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:36" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="D5" s="11"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="H5" s="16"/>
       <c r="I5" s="16">
         <v>45455</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
-      <c r="AC5" s="24">
+      <c r="AC5" s="23">
         <v>33</v>
       </c>
-      <c r="AD5" s="25"/>
+      <c r="AD5" s="24"/>
     </row>
     <row r="6" spans="1:36" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="D6" s="11"/>
-      <c r="AC6" s="24">
+      <c r="AC6" s="23">
         <v>33</v>
       </c>
-      <c r="AD6" s="25"/>
+      <c r="AD6" s="24"/>
     </row>
     <row r="7" spans="1:36" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
       <c r="D7" s="11"/>
-      <c r="AD7" s="25"/>
+      <c r="AD7" s="24"/>
     </row>
     <row r="8" spans="1:36" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11"/>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
       <c r="D8" s="11"/>
-      <c r="AD8" s="25"/>
+      <c r="AD8" s="24"/>
     </row>
     <row r="9" spans="1:36" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11"/>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
       <c r="D9" s="11"/>
-      <c r="AD9" s="25"/>
+      <c r="AD9" s="24"/>
     </row>
     <row r="10" spans="1:36" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11"/>
       <c r="B10" s="11"/>
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
-      <c r="AD10" s="25"/>
+      <c r="AD10" s="24"/>
     </row>
     <row r="11" spans="1:36" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11"/>
       <c r="B11" s="11"/>
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
-      <c r="AD11" s="25"/>
+      <c r="AD11" s="24"/>
     </row>
     <row r="12" spans="1:36" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11"/>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
       <c r="D12" s="11"/>
-      <c r="AD12" s="25"/>
+      <c r="AD12" s="24"/>
     </row>
     <row r="13" spans="1:36" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11"/>
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11"/>
-      <c r="AD13" s="25"/>
+      <c r="AD13" s="24"/>
     </row>
     <row r="14" spans="1:36" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11"/>
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
       <c r="D14" s="11"/>
-      <c r="AD14" s="25"/>
+      <c r="AD14" s="24"/>
     </row>
     <row r="15" spans="1:36" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11"/>
       <c r="B15" s="11"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11"/>
-      <c r="AD15" s="25"/>
+      <c r="AD15" s="24"/>
     </row>
     <row r="16" spans="1:36" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11"/>
       <c r="B16" s="11"/>
       <c r="C16" s="11"/>
       <c r="D16" s="11"/>
-      <c r="AD16" s="25"/>
+      <c r="AD16" s="24"/>
     </row>
     <row r="17" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11"/>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
       <c r="D17" s="11"/>
-      <c r="AD17" s="25"/>
+      <c r="AD17" s="24"/>
     </row>
     <row r="18" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11"/>
       <c r="B18" s="11"/>
       <c r="C18" s="11"/>
       <c r="D18" s="11"/>
-      <c r="AD18" s="25"/>
+      <c r="AD18" s="24"/>
     </row>
     <row r="19" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11"/>
       <c r="B19" s="11"/>
       <c r="C19" s="11"/>
       <c r="D19" s="11"/>
-      <c r="AD19" s="25"/>
+      <c r="AD19" s="24"/>
     </row>
     <row r="20" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11"/>
@@ -59721,7 +59708,7 @@
       <c r="D1008" s="11"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="21" type="noConversion"/>
+  <phoneticPr fontId="20" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B6" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"1. 主要,2. 次要,3. side - 主要,4. side - 次要,5. 沒有重要,6. 其它業務"</formula1>
@@ -59774,59 +59761,59 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F1" s="4">
         <v>2024</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J1" s="7"/>
       <c r="K1" s="7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="O1" s="8">
         <v>2025</v>
       </c>
       <c r="P1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="R1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="T1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="R1" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="T1" s="6" t="s">
-        <v>17</v>
-      </c>
       <c r="U1" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V1" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="X1" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="Y1" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="Z1" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AA1" s="6"/>
       <c r="AB1" s="6"/>
@@ -59836,16 +59823,16 @@
         <v>2026</v>
       </c>
       <c r="AF1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="AG1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="AH1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="AG1" s="3" t="s">
+      <c r="AI1" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="AH1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI1" s="3" t="s">
-        <v>9</v>
       </c>
       <c r="AJ1" s="6"/>
       <c r="AK1" s="6"/>
@@ -59856,64 +59843,64 @@
     </row>
     <row r="2" spans="1:41" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="9" t="s">
-        <v>21</v>
-      </c>
       <c r="C2" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F2" s="6"/>
       <c r="G2" s="6" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="J2" s="16"/>
       <c r="K2" s="16">
         <v>45455</v>
       </c>
       <c r="L2" s="11" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="M2" s="11" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="O2" s="11"/>
       <c r="P2" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q2" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="R2" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="T2" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="U2" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="V2" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="X2" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="Q2" s="11" t="s">
+      <c r="Y2" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="R2" s="11" t="s">
+      <c r="Z2" s="11" t="s">
         <v>41</v>
-      </c>
-      <c r="T2" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="U2" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="V2" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="X2" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y2" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="Z2" s="11" t="s">
-        <v>46</v>
       </c>
       <c r="AA2" s="11"/>
       <c r="AB2" s="11"/>
@@ -59935,25 +59922,25 @@
     </row>
     <row r="3" spans="1:41" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="9" t="s">
-        <v>21</v>
-      </c>
       <c r="C3" s="6" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="X3" s="21">
         <v>45938</v>
       </c>
       <c r="Y3" s="11" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="Z3" s="11" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="AA3" s="11"/>
       <c r="AB3" s="11"/>
@@ -59994,7 +59981,7 @@
       <c r="AO4" s="11"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="21" type="noConversion"/>
+  <phoneticPr fontId="20" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B3" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"1. 主要,2. 次要,3. side - 主要,4. side - 次要,5. 沒有重要,6. 其它業務"</formula1>
@@ -60014,16 +60001,15 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AL20"/>
+  <dimension ref="A1:AJ20"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="6" max="6" width="21.28515625" customWidth="1"/>
-    <col min="13" max="13" width="35.5703125" customWidth="1"/>
-    <col min="14" max="14" width="22.5703125" customWidth="1"/>
-    <col min="15" max="15" width="14.42578125" customWidth="1"/>
+    <col min="11" max="11" width="35.5703125" customWidth="1"/>
+    <col min="12" max="12" width="22.5703125" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:36" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -60036,16 +60022,16 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="2">
+        <v>2026</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="2">
-        <v>2026</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>6</v>
@@ -60053,19 +60039,15 @@
       <c r="K1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="1"/>
+      <c r="M1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="N1" s="1"/>
-      <c r="O1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="P1" s="3" t="s">
-        <v>12</v>
-      </c>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
@@ -60086,49 +60068,43 @@
       <c r="AH1" s="1"/>
       <c r="AI1" s="1"/>
       <c r="AJ1" s="1"/>
-      <c r="AK1" s="1"/>
-      <c r="AL1" s="1"/>
-    </row>
-    <row r="2" spans="1:38" ht="60.75" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:36" ht="60.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
-      <c r="D2" s="13" t="s">
-        <v>24</v>
+      <c r="D2" s="29" t="s">
+        <v>174</v>
       </c>
-      <c r="E2" s="13" t="s">
-        <v>31</v>
+      <c r="E2" s="11" t="s">
+        <v>33</v>
       </c>
-      <c r="F2" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="G2" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="16">
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="16">
         <v>46175</v>
       </c>
-      <c r="K2" s="19">
+      <c r="I2" s="19">
         <v>5</v>
       </c>
-      <c r="L2" s="20">
+      <c r="J2" s="20">
         <v>374.72</v>
       </c>
+      <c r="K2" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="L2" s="11"/>
       <c r="M2" s="11" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="N2" s="11"/>
-      <c r="O2" s="11" t="s">
-        <v>48</v>
-      </c>
+      <c r="O2" s="11"/>
       <c r="P2" s="11"/>
       <c r="Q2" s="11"/>
       <c r="R2" s="11"/>
@@ -60150,34 +60126,30 @@
       <c r="AH2" s="11"/>
       <c r="AI2" s="11"/>
       <c r="AJ2" s="11"/>
-      <c r="AK2" s="11"/>
-      <c r="AL2" s="11"/>
-    </row>
-    <row r="3" spans="1:38" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:36" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
-      <c r="E3" s="17"/>
-      <c r="F3" s="23" t="s">
-        <v>71</v>
+      <c r="E3" s="11" t="s">
+        <v>33</v>
       </c>
-      <c r="G3" s="11" t="s">
-        <v>38</v>
-      </c>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
       <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="20"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11"/>
       <c r="M3" s="11"/>
       <c r="N3" s="11"/>
       <c r="O3" s="11"/>
@@ -60202,62 +60174,60 @@
       <c r="AH3" s="11"/>
       <c r="AI3" s="11"/>
       <c r="AJ3" s="11"/>
-      <c r="AK3" s="11"/>
-      <c r="AL3" s="11"/>
-    </row>
-    <row r="4" spans="1:38" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L4" s="25"/>
-    </row>
-    <row r="5" spans="1:38" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L5" s="25"/>
-    </row>
-    <row r="6" spans="1:38" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L6" s="25"/>
-    </row>
-    <row r="7" spans="1:38" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L7" s="25"/>
-    </row>
-    <row r="8" spans="1:38" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L8" s="25"/>
-    </row>
-    <row r="9" spans="1:38" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L9" s="25"/>
-    </row>
-    <row r="10" spans="1:38" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L10" s="25"/>
-    </row>
-    <row r="11" spans="1:38" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L11" s="25"/>
-    </row>
-    <row r="12" spans="1:38" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L12" s="25"/>
-    </row>
-    <row r="13" spans="1:38" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L13" s="25"/>
-    </row>
-    <row r="14" spans="1:38" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L14" s="25"/>
-    </row>
-    <row r="15" spans="1:38" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L15" s="25"/>
-    </row>
-    <row r="16" spans="1:38" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L16" s="25"/>
-    </row>
-    <row r="17" spans="12:12" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L17" s="25"/>
-    </row>
-    <row r="18" spans="12:12" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L18" s="25"/>
-    </row>
-    <row r="19" spans="12:12" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L19" s="25"/>
-    </row>
-    <row r="20" spans="12:12" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="L20" s="25"/>
+    </row>
+    <row r="4" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J4" s="24"/>
+    </row>
+    <row r="5" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J5" s="24"/>
+    </row>
+    <row r="6" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J6" s="24"/>
+    </row>
+    <row r="7" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J7" s="24"/>
+    </row>
+    <row r="8" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J8" s="24"/>
+    </row>
+    <row r="9" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J9" s="24"/>
+    </row>
+    <row r="10" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J10" s="24"/>
+    </row>
+    <row r="11" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J11" s="24"/>
+    </row>
+    <row r="12" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J12" s="24"/>
+    </row>
+    <row r="13" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J13" s="24"/>
+    </row>
+    <row r="14" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J14" s="24"/>
+    </row>
+    <row r="15" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J15" s="24"/>
+    </row>
+    <row r="16" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J16" s="24"/>
+    </row>
+    <row r="17" spans="10:10" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J17" s="24"/>
+    </row>
+    <row r="18" spans="10:10" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J18" s="24"/>
+    </row>
+    <row r="19" spans="10:10" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J19" s="24"/>
+    </row>
+    <row r="20" spans="10:10" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="J20" s="24"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="21" type="noConversion"/>
+  <phoneticPr fontId="20" type="noConversion"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B3" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"1. 主要,2. 次要,3. side - 主要,4. side - 次要,5. 沒有重要,6. 其它業務"</formula1>
@@ -60268,12 +60238,9 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
-    <hyperlink ref="E2" r:id="rId2" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
-    <hyperlink ref="F2" r:id="rId3" xr:uid="{00000000-0004-0000-0300-000002000000}"/>
-    <hyperlink ref="D3" r:id="rId4" xr:uid="{00000000-0004-0000-0300-000003000000}"/>
-    <hyperlink ref="F3" r:id="rId5" xr:uid="{00000000-0004-0000-0300-000004000000}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{00000000-0004-0000-0300-000003000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId6"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>